<commit_message>
Fase 142: Llamadas Únicas rechaza SKILL_NAME = NO CONTESTADAS (v1.33.1)
Una sola fila NO CONTESTADAS hace que la hoja completa quede con error en
la vista previa ("NO CONTESTADAS es una llamada de SALIDA no conectada;
cárgala en Llamadas de salida.") y no se guarde. El servidor sigue
aceptando ABANDONADA para cuando haya fuente real de abandonadas
entrantes. Plantilla sin el ejemplo NO CONTESTADAS. Pruebas
actualizadas (sin debilitar) y nueva; guía, CHANGELOG, pendientes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_LLAMADAS_UNICAS_MOBILIZE.xlsx
+++ b/server/plantillas/PLANTILLA_LLAMADAS_UNICAS_MOBILIZE.xlsx
@@ -397,13 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,23 +427,9 @@
         <v>SKILL SAC</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Asesor Ejemplo</v>
-      </c>
-      <c r="B3" t="str">
-        <v>02/09/2026</v>
-      </c>
-      <c r="C3" t="str">
-        <v>3000000001</v>
-      </c>
-      <c r="D3" t="str">
-        <v>NO CONTESTADAS</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>